<commit_message>
feat(Colorfull): đổi bảng màu theo tệp mẫu người dùng chỉnh lại (2026-09-23)
Nguồn: "Copy of Copy of E2E_-_Nhap_tu_Excel_091-new4.xlsx" bản sửa sáng 2026-09-23.
- Hàng nhóm F6D479 → F4CFB0, nhóm con D5DDA2 → CAD8AA (cấu hình + màn hình soạn).
- Nền nướng sẵn trong CLF_KhongNgay/CLF_CoNgay: dải tiêu đề 9CCDC9 chữ 243139,
  tiêu đề cột + khối tổng 9DCCC9 (trước là theme8 tint 0.4). Script: scripts/doi-mau-clf.mjs.
- excelImport vẫn nhận F6D479/D5DDA2 của tệp đã gửi khách hôm trước.
- Snapshot clf đổi: đối chiếu từng ô, khác 25/109 ô, tất cả chỉ là màu.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/CLF_CoNgay.xlsx
+++ b/templates/CLF_CoNgay.xlsx
@@ -341,7 +341,7 @@
     </font>
     <font>
       <b/>
-      <color theme="1"/>
+      <color rgb="FF243139"/>
       <family val="1"/>
       <sz val="18"/>
       <name val="Times New Roman"/>
@@ -459,7 +459,7 @@
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -468,14 +468,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999755851924192"/>
+        <fgColor rgb="FF9CCDC9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9DCCC9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.3999755851924192"/>
-        <bgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -648,22 +654,22 @@
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -726,7 +732,7 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">

</xml_diff>